<commit_message>
feat: add storage functionality for finalized scales
Implement saving, loading, and deletion of distribution lists, updating storage keys and enhancing the EscalaFinalTab and DistribuicaoTab interfaces to support scale persistence.
</commit_message>
<xml_diff>
--- a/public/modelos/Modelo_Lista_DEJEP_Policial.xlsx
+++ b/public/modelos/Modelo_Lista_DEJEP_Policial.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,22 +442,62 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>5. A coluna "Limite Max DEJEP" indica a quantidade máxima de diárias que o policial aceita (padrão 8).</v>
+        <v>5. REGRAS OBRIGATÓRIAS DOS TURNOS:</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6. Status deve ser "Apto" para participar da distribuição.</v>
+        <v xml:space="preserve">   - Policial do Turno I pode fazer DEJEP nos turnos II, III e IV (não no Turno I).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v xml:space="preserve">   - Policial do Turno II pode fazer DEJEP nos turnos I, III e IV (não no Turno II).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v xml:space="preserve">   - Policial do Turno III pode fazer DEJEP nos turnos I, II e IV (não no Turno III).</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v xml:space="preserve">   - Policial do Turno IV pode fazer DEJEP nos turnos I, II e III (não no Turno IV).</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v xml:space="preserve">   - Policial Diarista (expediente comercial seg-sex 07h-16h) pode fazer DEJEP:</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">       * Nos Turnos II e IV (noturnos): APENAS às sextas-feiras e aos sábados.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v xml:space="preserve">       * Nos Turnos I e III (diurnos): APENAS aos sábados e domingos.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>6. A coluna "Limite Max DEJEP" indica a quantidade máxima de diárias que o policial aceita (padrão 8).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>7. Status deve ser "Apto" para participar da distribuição.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -512,10 +552,10 @@
         <v>Policial Penal - Classe Especial</v>
       </c>
       <c r="E2" t="str">
-        <v>Turno 1 (Alfa)</v>
+        <v>Turno I (Diurno)</v>
       </c>
       <c r="F2" t="str">
-        <v>02/11/2026, 04/11/2026, 07/11/2026, 09/11/2026, 11/11/2026, 14/11/2026, 18/11/2026, 21/11/2026</v>
+        <v>01/11/2026, 03/11/2026, 05/11/2026, 08/11/2026, 10/11/2026, 15/11/2026, 17/11/2026, 22/11/2026</v>
       </c>
       <c r="G2">
         <v>8</v>
@@ -544,10 +584,10 @@
         <v>Policial Penal - Classe II</v>
       </c>
       <c r="E3" t="str">
-        <v>Turno 2 (Bravo)</v>
+        <v>Turno II (Noturno)</v>
       </c>
       <c r="F3" t="str">
-        <v>01/11/2026, 03/11/2026, 05/11/2026, 08/11/2026, 12/11/2026, 15/11/2026, 19/11/2026, 24/11/2026, 29/11/2026</v>
+        <v>02/11/2026, 04/11/2026, 06/11/2026, 07/11/2026, 11/11/2026, 14/11/2026, 18/11/2026, 21/11/2026, 28/11/2026</v>
       </c>
       <c r="G3">
         <v>9</v>
@@ -576,10 +616,10 @@
         <v>Policial Penal - Classe I</v>
       </c>
       <c r="E4" t="str">
-        <v>Turno 3 (Charlie)</v>
+        <v>Turno III (Diurno)</v>
       </c>
       <c r="F4" t="str">
-        <v>02/11/2026, 06/11/2026, 07/11/2026, 13/11/2026, 16/11/2026, 20/11/2026, 27/11/2026</v>
+        <v>01/11/2026, 05/11/2026, 08/11/2026, 12/11/2026, 15/11/2026, 22/11/2026, 29/11/2026</v>
       </c>
       <c r="G4">
         <v>7</v>
@@ -608,10 +648,10 @@
         <v>Policial Penal - Classe II</v>
       </c>
       <c r="E5" t="str">
-        <v>Turno 4 (Delta)</v>
+        <v>Turno IV (Noturno)</v>
       </c>
       <c r="F5" t="str">
-        <v>01/11/2026, 07/11/2026, 08/11/2026, 14/11/2026, 15/11/2026, 21/11/2026, 22/11/2026, 28/11/2026, 29/11/2026, 30/11/2026</v>
+        <v>02/11/2026, 04/11/2026, 06/11/2026, 09/11/2026, 11/11/2026, 13/11/2026, 16/11/2026, 18/11/2026, 23/11/2026, 25/11/2026</v>
       </c>
       <c r="G5">
         <v>10</v>
@@ -640,13 +680,13 @@
         <v>Policial Penal - Classe I</v>
       </c>
       <c r="E6" t="str">
-        <v>Administrativo</v>
+        <v>Diaristas</v>
       </c>
       <c r="F6" t="str">
-        <v>03/11/2026, 05/11/2026, 10/11/2026, 12/11/2026, 17/11/2026, 19/11/2026</v>
+        <v>01/11/2026, 06/11/2026, 07/11/2026, 08/11/2026, 13/11/2026, 14/11/2026, 15/11/2026, 21/11/2026</v>
       </c>
       <c r="G6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H6">
         <v>6</v>
@@ -672,10 +712,10 @@
         <v>Policial Penal - Classe Especial</v>
       </c>
       <c r="E7" t="str">
-        <v>Turno 1 (Alfa)</v>
+        <v>Turno I (Diurno)</v>
       </c>
       <c r="F7" t="str">
-        <v>04/11/2026, 06/11/2026, 11/11/2026, 13/11/2026, 18/11/2026, 20/11/2026, 25/11/2026</v>
+        <v>03/11/2026, 05/11/2026, 10/11/2026, 12/11/2026, 17/11/2026, 19/11/2026, 24/11/2026</v>
       </c>
       <c r="G7">
         <v>7</v>
@@ -704,10 +744,10 @@
         <v>Policial Penal - Classe Especial</v>
       </c>
       <c r="E8" t="str">
-        <v>Turno 3 (Charlie)</v>
+        <v>Turno III (Diurno)</v>
       </c>
       <c r="F8" t="str">
-        <v>02/11/2026, 07/11/2026, 09/11/2026, 14/11/2026, 21/11/2026</v>
+        <v>01/11/2026, 07/11/2026, 08/11/2026, 15/11/2026, 22/11/2026</v>
       </c>
       <c r="G8">
         <v>5</v>

</xml_diff>